<commit_message>
Stage 8 fixes: F-015
</commit_message>
<xml_diff>
--- a/output/archive/DurnesswickData/Admin/Finance/2025/early-CMC_rates_041525_revB.xlsx
+++ b/output/archive/DurnesswickData/Admin/Finance/2025/early-CMC_rates_041525_revB.xlsx
@@ -499,22 +499,20 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Vehicle ladder work package</t>
+          <t>Vehicle ladder</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>per work package</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Quoted at scoping</t>
-        </is>
+          <t>per vehicle ladder</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>10900</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Two-week screen with bench sheet per vehicle</t>
+          <t>Two-week screen with bench sheet per vehicle. No volume discount</t>
         </is>
       </c>
     </row>
@@ -588,7 +586,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Rates are set at scoping against the work package. This card does not commit a price for a formulation set that has not been scoped.</t>
+          <t>The Vehicle ladder rate is the 2025 list price. Other lines are quoted at scoping against the work package, and this card does not commit a price for a formulation set that has not been scoped.</t>
         </is>
       </c>
     </row>

</xml_diff>